<commit_message>
fixes as per the provided md file
</commit_message>
<xml_diff>
--- a/02_ai-risk-framework-implementation-nist-ai-rmf/demo/risk_assessment_demo.xlsx
+++ b/02_ai-risk-framework-implementation-nist-ai-rmf/demo/risk_assessment_demo.xlsx
@@ -1006,34 +1006,34 @@
       <c r="B5" s="23" t="inlineStr">
         <is>
           <t>"Manage"
-Reasoning: System downtime requires active MANAGEMENT — deploying redundancy, failover mechanisms, and operational procedures. Infrastructure resilience is a management task.</t>
+Reasoning: Incident response is an active MANAGEMENT control — building playbooks, escalation paths and on-call rotations to respond when DiagnosAI fails.</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Technical</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>System downtime during critical care: DiagnosAI unavailability during peak ER hours forces clinicians to operate without decision support</t>
+          <t>Incident response gap: Inadequate procedures to respond to DiagnosAI failures or adverse events</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>IT Infrastructure Manager</t>
+          <t>Chief Medical Officer</t>
         </is>
       </c>
       <c r="F5" s="23" t="inlineStr">
         <is>
           <t>"4"
-Reasoning: Impact=4 (High): ER physicians rely on DiagnosAI for decision support during peak hours. Downtime means operating without AI assistance — increased cognitive load and potential for errors.</t>
+Reasoning: Impact=4 (High): an unhandled DiagnosAI failure in the ER delays care and can harm patients.</t>
         </is>
       </c>
       <c r="G5" s="23" t="inlineStr">
         <is>
           <t>"3"
-Reasoning: Likelihood=3 (Moderate): System outages happen in any environment. Peak ER hours create maximum demand. Moderate probability within 12 months.</t>
+Reasoning: Likelihood=3 (Moderate): failures and adverse events occur in any clinical AI deployment.</t>
         </is>
       </c>
       <c r="H5" s="23" t="n">
@@ -1046,14 +1046,14 @@
       </c>
       <c r="J5" s="23" t="inlineStr">
         <is>
-          <t>"Deploy redundant systems with geographic distribution, implement failover mechanisms, establish manual fallback protocols, conduct quarterly disaster recovery drills"
-Reasoning: Geographic distribution prevents single-site failures. Failover is automatic. Manual fallback ensures care continues without AI. DR drills verify everything works under stress.</t>
+          <t>"Develop incident response playbook with clear escalation paths; establish on-call response rotation; run tabletop exercises against DiagnosAI failure scenarios"
+Reasoning: A documented playbook plus a named on-call path converts an ad-hoc reaction into a repeatable control.</t>
         </is>
       </c>
       <c r="K5" s="23" t="inlineStr">
         <is>
           <t>"High"
-Reasoning: Score 12 = High. In an ER, any downtime is potentially dangerous. 30-day mitigation timeline appropriate.</t>
+Reasoning: Score 12 = High. Gaps in incident response amplify every other failure mode.</t>
         </is>
       </c>
       <c r="L5" s="14" t="inlineStr">

</xml_diff>